<commit_message>
Add advanced after-tax NPV mode (capex/opex, Section 174A amortization, tax shield, discounting)
</commit_message>
<xml_diff>
--- a/build-buy-automate-tco-calculator.xlsx
+++ b/build-buy-automate-tco-calculator.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculator" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advanced (After-Tax NPV)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +71,12 @@
       <b val="1"/>
       <color rgb="0024292F"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008250DF"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -199,7 +206,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -264,6 +271,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -272,6 +282,30 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -638,11 +672,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B30"/>
+  <dimension ref="B2:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="102" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -655,164 +689,271 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Companion to Engineering Economics, Part 5. A working five-year total-cost-of-ownership model.</t>
+          <t>Companion to Engineering Economics, Part 5. A working total-cost-of-ownership model.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>How to use this</t>
+          <t>Two ways to use this workbook</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>1. Open the 'Calculator' tab.</t>
+          <t>SIMPLE (tabs: 'Calculator' and 'Sensitivity')</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2. Edit only the shaded blue cells. Those are your assumptions. Everything else is a formula.</t>
+          <t xml:space="preserve">   Plain five-year cash totals. Enter costs, read the winner. Ten minutes, no finance background needed.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>3. Read the five-year totals and the winner at the bottom. Change an assumption and watch them move.</t>
+          <t xml:space="preserve">   Start here. For many decisions this is all you need.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>4. Use the 'Sensitivity' tab to see whether the decision flips when maintenance is cheaper or more expensive.</t>
-        </is>
-      </c>
+      <c r="B9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>ADVANCED (tab: 'Advanced (After-Tax NPV)')</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>The one idea this model exists to enforce</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Same decision, but modeled the way a CFO sees it: capital vs. operating expense, amortization,</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Initial development is roughly 20% of a system's lifetime cost. Maintenance is the other 60-80%.</t>
+          <t xml:space="preserve">   the tax shield, and discounting to present value. Use it when the dollar amounts are large enough</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>A build estimate that stops at 'one quarter' has priced about a fifth of the real total. This</t>
+          <t xml:space="preserve">   that accounting treatment and the time value of money actually change the ranking.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>model forces the other four-fifths onto the page by making you enter a yearly maintenance number</t>
-        </is>
-      </c>
+      <c r="B14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>and multiplying it across the time horizon.</t>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>How to use the SIMPLE tabs</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>1. On 'Calculator', edit only the shaded blue cells. Everything else is a formula.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>The three columns</t>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>2. Read the five-year totals and the auto-selected winner at the bottom.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>BUILD    - you build it on open source / in-house. Low or zero license, high maintenance.</t>
+          <t>3. On 'Sensitivity', see whether the winner flips when BUILD maintenance is cheaper or costlier.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>BUY      - you license a product. The fee is visible; integration and renewal escalation are not.</t>
-        </is>
-      </c>
+      <c r="B19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>AUTOMATE - you script around the need with tools you already run. Cheapest, but often covers less.</t>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>How to use the ADVANCED tab</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="4" t="inlineStr"/>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>1. It pulls your cost inputs straight from the 'Calculator' tab, so fill that in first.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Honest limits (read these)</t>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>2. Then set the finance assumptions in the blue cells: tax rate, discount rate, and the</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>- The maintenance figure drives the whole result and is the hardest to predict. Use the Sensitivity tab.</t>
+          <t xml:space="preserve">   amortization period for capitalized build cost (US Section 174 default is 5 years).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>- This models cost, not value or capability. Automate is cheapest here precisely because it often does less.</t>
+          <t>3. Read two bottom-line numbers per option: nominal five-year cash, and after-tax NPV.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>- Loaded cost means salary + benefits + payroll tax + equipment + overhead, not base salary.</t>
+          <t xml:space="preserve">   The after-tax NPV is the number a finance team actually decides on.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>- Don't build a five-year model to decide on a $50/month tool. Use it for large, durable, hard-to-reverse calls.</t>
-        </is>
-      </c>
+      <c r="B26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="B27" s="4" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Why accounting treatment changes the answer</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>Cash out the door is not the same as cost after tax. A deduction you take this year is worth more</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>than the same deduction spread over several years, because money now beats money later. US tax</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>treatment of software R&amp;D has moved: capitalize-and-amortize over 5 years applied 2022-2024, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>the 2025 OBBBA (Section 174A) restored immediate expensing for domestic R&amp;D while foreign work</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>still amortizes over 15 years. Set the amortization period cell to match your situation (1 = expense</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>now). A SaaS subscription is usually a clean operating expense deducted right away. Where build</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>labor lands on that line tilts build vs. buy, and the SIMPLE cash model cannot see it. ADVANCED can.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>IMPORTANT: this is a model, not tax advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Section 174, bonus depreciation, and capitalization rules change with legislation and vary by</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>jurisdiction and company. Every tax assumption here is an editable blue cell with an illustrative</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>default. Confirm the treatment with your own finance and tax team before you decide anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>The one idea the whole thing exists to enforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Initial development is roughly 20% of a system's lifetime cost. Maintenance is the other 60-80%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>A build estimate that stops at 'one quarter' has priced about a fifth of the real total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
           <t>Default numbers are illustrative, from the article. Replace every blue cell with your own.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="5" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Blue cells = your inputs. Edit these.</t>
         </is>
@@ -829,7 +970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -842,14 +983,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Five-Year TCO Calculator</t>
+          <t>Five-Year TCO Calculator (Simple)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Edit the blue cells. Totals recalculate automatically.</t>
+          <t>Plain cash totals. Edit the blue cells; totals recalculate automatically.</t>
         </is>
       </c>
     </row>
@@ -1131,18 +1272,26 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="25" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>Want taxes, capex/opex, and present value? See the 'Advanced (After-Tax NPV)' tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="inlineStr">
         <is>
           <t>Default values are illustrative, from the article. Replace every blue cell with your own numbers.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A26:D26"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="B22:D22"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1174,54 +1323,34 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="25" t="inlineStr">
         <is>
-          <t>The maintenance assumption drives the result and is the hardest to predict. This sweeps BUILD maintenance effort and recomputes the five-year totals, holding the Calculator's other inputs fixed. If the winner changes across the rows, maintenance is the assumption that actually matters: spend your estimation effort there.</t>
+          <t>The maintenance assumption drives the result and is the hardest to predict. This sweeps BUILD maintenance effort and recomputes the five-year totals, holding the Calculator's other inputs fixed. If the winner changes across the rows, maintenance is the assumption that matters most.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>BUILD maintenance (FTE)</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>BUILD 5-yr total</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>BUY 5-yr total</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>AUTOMATE 5-yr total</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Lowest cost</t>
-        </is>
-      </c>
+      <c r="A4" s="12" t="n"/>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="12" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
         <v>0.1</v>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="27">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A5*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="27">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="27">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B5:D5),B5:D5,0))</f>
         <v/>
       </c>
@@ -1230,19 +1359,19 @@
       <c r="A6" s="9" t="n">
         <v>0.25</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="29">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A6*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="29">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D6" s="28">
+      <c r="D6" s="29">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B6:D6),B6:D6,0))</f>
         <v/>
       </c>
@@ -1251,19 +1380,19 @@
       <c r="A7" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="27">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A7*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="27">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="27">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B7:D7),B7:D7,0))</f>
         <v/>
       </c>
@@ -1272,19 +1401,19 @@
       <c r="A8" s="9" t="n">
         <v>0.75</v>
       </c>
-      <c r="B8" s="28">
+      <c r="B8" s="29">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A8*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C8" s="28">
+      <c r="C8" s="29">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D8" s="28">
+      <c r="D8" s="29">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B8:D8),B8:D8,0))</f>
         <v/>
       </c>
@@ -1293,19 +1422,19 @@
       <c r="A9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="26">
+      <c r="B9" s="27">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A9*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="27">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="27">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B9:D9),B9:D9,0))</f>
         <v/>
       </c>
@@ -1314,19 +1443,19 @@
       <c r="A10" s="9" t="n">
         <v>1.5</v>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="29">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A10*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="29">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="29">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E10" s="27">
+      <c r="E10" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B10:D10),B10:D10,0))</f>
         <v/>
       </c>
@@ -1335,19 +1464,19 @@
       <c r="A11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="26">
+      <c r="B11" s="27">
         <f>(Calculator!$B$9+Calculator!$B$16+Calculator!$B$18)+A11*Calculator!$B$6*Calculator!$B$5</f>
         <v/>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="27">
         <f>Calculator!$C$19</f>
         <v/>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="27">
         <f>Calculator!$D$19</f>
         <v/>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="28">
         <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B11:D11),B11:D11,0))</f>
         <v/>
       </c>
@@ -1366,4 +1495,819 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Advanced: After-Tax NPV</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="56" customHeight="1">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>The same decision a CFO's way: capital vs. operating expense, amortization, the tax shield, and present value. Cost inputs come from the 'Calculator' tab (fill that in first). Set the finance assumptions in the blue cells below. NOT TAX ADVICE: confirm treatment with your finance team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Finance assumptions (edit these)</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Marginal tax rate (%)</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Discount rate / WACC (%)</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Build amortization period (years; 1 = expense now)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>US domestic R&amp;D is expensable now (set 1); 5 = 2022-24 rule / an election; foreign = 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Treat BUILD initial cost as capex? (1=yes,0=no)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Treat BUY integration as capex? (1=yes,0=no)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Treat AUTOMATE setup as capex? (1=yes,0=no)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Per-year after-tax cash flow (up to 10 years shown; years beyond your horizon are zero).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>BUILD</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="17">
+        <f>(IF(1=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((1&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(1-1),0))+(IF((1&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C16" s="17">
+        <f>((IF((1&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(1-1),0))+(IF((1&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(1&gt;=1,1&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(1=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D16" s="17">
+        <f>(B16-$B$5*C16)/((1+$B$6)^1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="17">
+        <f>(IF(2=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((2&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(2-1),0))+(IF((2&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C17" s="17">
+        <f>((IF((2&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(2-1),0))+(IF((2&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(2&gt;=1,2&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(2=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D17" s="17">
+        <f>(B17-$B$5*C17)/((1+$B$6)^2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="17">
+        <f>(IF(3=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((3&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(3-1),0))+(IF((3&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C18" s="17">
+        <f>((IF((3&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(3-1),0))+(IF((3&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(3&gt;=1,3&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(3=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D18" s="17">
+        <f>(B18-$B$5*C18)/((1+$B$6)^3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="17">
+        <f>(IF(4=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((4&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(4-1),0))+(IF((4&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C19" s="17">
+        <f>((IF((4&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(4-1),0))+(IF((4&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(4&gt;=1,4&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(4=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D19" s="17">
+        <f>(B19-$B$5*C19)/((1+$B$6)^4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B20" s="17">
+        <f>(IF(5=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((5&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(5-1),0))+(IF((5&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C20" s="17">
+        <f>((IF((5&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(5-1),0))+(IF((5&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(5&gt;=1,5&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(5=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D20" s="17">
+        <f>(B20-$B$5*C20)/((1+$B$6)^5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B21" s="17">
+        <f>(IF(6=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((6&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(6-1),0))+(IF((6&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C21" s="17">
+        <f>((IF((6&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(6-1),0))+(IF((6&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(6&gt;=1,6&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(6=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D21" s="17">
+        <f>(B21-$B$5*C21)/((1+$B$6)^6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="17">
+        <f>(IF(7=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((7&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(7-1),0))+(IF((7&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C22" s="17">
+        <f>((IF((7&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(7-1),0))+(IF((7&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(7&gt;=1,7&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(7=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D22" s="17">
+        <f>(B22-$B$5*C22)/((1+$B$6)^7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="17">
+        <f>(IF(8=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((8&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(8-1),0))+(IF((8&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C23" s="17">
+        <f>((IF((8&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(8-1),0))+(IF((8&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(8&gt;=1,8&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(8=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>(B23-$B$5*C23)/((1+$B$6)^8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B24" s="17">
+        <f>(IF(9=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((9&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(9-1),0))+(IF((9&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C24" s="17">
+        <f>((IF((9&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(9-1),0))+(IF((9&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(9&gt;=1,9&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(9=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D24" s="17">
+        <f>(B24-$B$5*C24)/((1+$B$6)^9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B25" s="17">
+        <f>(IF(10=1,Calculator!$B$9+Calculator!$B$13*Calculator!$B$14,0))+(IF((10&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(10-1),0))+(IF((10&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C25" s="17">
+        <f>((IF((10&lt;=Calculator!$B$5),Calculator!$B$10*(1+Calculator!$B$11)^(10-1),0))+(IF((10&lt;=Calculator!$B$5),Calculator!$B$12*Calculator!$B$6,0)))+(IF(AND(10&gt;=1,10&lt;=$B$7),Calculator!$B$9*$B$8/$B$7,0))+(IF(10=1,Calculator!$B$9*(1-$B$8)+Calculator!$B$13*Calculator!$B$14,0))</f>
+        <v/>
+      </c>
+      <c r="D25" s="17">
+        <f>(B25-$B$5*C25)/((1+$B$6)^10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>NPV of after-tax cost</t>
+        </is>
+      </c>
+      <c r="B26" s="17">
+        <f>SUM(B16:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>(nominal cash &lt;-)</t>
+        </is>
+      </c>
+      <c r="D26" s="34">
+        <f>SUM(D16:D25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="n"/>
+      <c r="C28" s="36" t="n"/>
+      <c r="D28" s="36" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="17">
+        <f>(IF(1=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((1&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(1-1),0))+(IF((1&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C30" s="17">
+        <f>((IF((1&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(1-1),0))+(IF((1&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(1&gt;=1,1&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(1=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D30" s="17">
+        <f>(B30-$B$5*C30)/((1+$B$6)^1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="17">
+        <f>(IF(2=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((2&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(2-1),0))+(IF((2&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C31" s="17">
+        <f>((IF((2&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(2-1),0))+(IF((2&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(2&gt;=1,2&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(2=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D31" s="17">
+        <f>(B31-$B$5*C31)/((1+$B$6)^2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="17">
+        <f>(IF(3=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((3&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(3-1),0))+(IF((3&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C32" s="17">
+        <f>((IF((3&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(3-1),0))+(IF((3&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(3&gt;=1,3&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(3=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D32" s="17">
+        <f>(B32-$B$5*C32)/((1+$B$6)^3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="17">
+        <f>(IF(4=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((4&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(4-1),0))+(IF((4&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C33" s="17">
+        <f>((IF((4&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(4-1),0))+(IF((4&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(4&gt;=1,4&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(4=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D33" s="17">
+        <f>(B33-$B$5*C33)/((1+$B$6)^4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="17">
+        <f>(IF(5=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((5&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(5-1),0))+(IF((5&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C34" s="17">
+        <f>((IF((5&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(5-1),0))+(IF((5&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(5&gt;=1,5&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(5=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D34" s="17">
+        <f>(B34-$B$5*C34)/((1+$B$6)^5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="17">
+        <f>(IF(6=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((6&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(6-1),0))+(IF((6&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C35" s="17">
+        <f>((IF((6&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(6-1),0))+(IF((6&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(6&gt;=1,6&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(6=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D35" s="17">
+        <f>(B35-$B$5*C35)/((1+$B$6)^6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B36" s="17">
+        <f>(IF(7=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((7&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(7-1),0))+(IF((7&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C36" s="17">
+        <f>((IF((7&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(7-1),0))+(IF((7&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(7&gt;=1,7&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(7=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D36" s="17">
+        <f>(B36-$B$5*C36)/((1+$B$6)^7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" s="17">
+        <f>(IF(8=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((8&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(8-1),0))+(IF((8&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C37" s="17">
+        <f>((IF((8&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(8-1),0))+(IF((8&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(8&gt;=1,8&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(8=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D37" s="17">
+        <f>(B37-$B$5*C37)/((1+$B$6)^8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B38" s="17">
+        <f>(IF(9=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((9&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(9-1),0))+(IF((9&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C38" s="17">
+        <f>((IF((9&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(9-1),0))+(IF((9&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(9&gt;=1,9&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(9=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D38" s="17">
+        <f>(B38-$B$5*C38)/((1+$B$6)^9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B39" s="17">
+        <f>(IF(10=1,Calculator!$C$9+Calculator!$C$13*Calculator!$C$14,0))+(IF((10&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(10-1),0))+(IF((10&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C39" s="17">
+        <f>((IF((10&lt;=Calculator!$B$5),Calculator!$C$10*(1+Calculator!$C$11)^(10-1),0))+(IF((10&lt;=Calculator!$B$5),Calculator!$C$12*Calculator!$B$6,0)))+(IF(AND(10&gt;=1,10&lt;=$B$7),Calculator!$C$9*$B$9/$B$7,0))+(IF(10=1,Calculator!$C$9*(1-$B$9)+Calculator!$C$13*Calculator!$C$14,0))</f>
+        <v/>
+      </c>
+      <c r="D39" s="17">
+        <f>(B39-$B$5*C39)/((1+$B$6)^10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>NPV of after-tax cost</t>
+        </is>
+      </c>
+      <c r="B40" s="17">
+        <f>SUM(B30:B39)</f>
+        <v/>
+      </c>
+      <c r="C40" s="33" t="inlineStr">
+        <is>
+          <t>(nominal cash &lt;-)</t>
+        </is>
+      </c>
+      <c r="D40" s="34">
+        <f>SUM(D30:D39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="37" t="inlineStr">
+        <is>
+          <t>AUTOMATE</t>
+        </is>
+      </c>
+      <c r="B42" s="38" t="n"/>
+      <c r="C42" s="38" t="n"/>
+      <c r="D42" s="38" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="n"/>
+      <c r="B43" s="12" t="n"/>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="17">
+        <f>(IF(1=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((1&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(1-1),0))+(IF((1&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C44" s="17">
+        <f>((IF((1&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(1-1),0))+(IF((1&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(1&gt;=1,1&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(1=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D44" s="17">
+        <f>(B44-$B$5*C44)/((1+$B$6)^1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="17">
+        <f>(IF(2=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((2&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(2-1),0))+(IF((2&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C45" s="17">
+        <f>((IF((2&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(2-1),0))+(IF((2&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(2&gt;=1,2&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(2=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D45" s="17">
+        <f>(B45-$B$5*C45)/((1+$B$6)^2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="17">
+        <f>(IF(3=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((3&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(3-1),0))+(IF((3&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C46" s="17">
+        <f>((IF((3&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(3-1),0))+(IF((3&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(3&gt;=1,3&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(3=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D46" s="17">
+        <f>(B46-$B$5*C46)/((1+$B$6)^3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="17">
+        <f>(IF(4=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((4&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(4-1),0))+(IF((4&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C47" s="17">
+        <f>((IF((4&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(4-1),0))+(IF((4&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(4&gt;=1,4&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(4=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D47" s="17">
+        <f>(B47-$B$5*C47)/((1+$B$6)^4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" s="17">
+        <f>(IF(5=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((5&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(5-1),0))+(IF((5&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C48" s="17">
+        <f>((IF((5&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(5-1),0))+(IF((5&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(5&gt;=1,5&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(5=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D48" s="17">
+        <f>(B48-$B$5*C48)/((1+$B$6)^5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" s="17">
+        <f>(IF(6=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((6&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(6-1),0))+(IF((6&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C49" s="17">
+        <f>((IF((6&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(6-1),0))+(IF((6&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(6&gt;=1,6&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(6=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D49" s="17">
+        <f>(B49-$B$5*C49)/((1+$B$6)^6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B50" s="17">
+        <f>(IF(7=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((7&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(7-1),0))+(IF((7&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C50" s="17">
+        <f>((IF((7&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(7-1),0))+(IF((7&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(7&gt;=1,7&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(7=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D50" s="17">
+        <f>(B50-$B$5*C50)/((1+$B$6)^7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="B51" s="17">
+        <f>(IF(8=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((8&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(8-1),0))+(IF((8&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C51" s="17">
+        <f>((IF((8&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(8-1),0))+(IF((8&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(8&gt;=1,8&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(8=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D51" s="17">
+        <f>(B51-$B$5*C51)/((1+$B$6)^8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" s="17">
+        <f>(IF(9=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((9&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(9-1),0))+(IF((9&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C52" s="17">
+        <f>((IF((9&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(9-1),0))+(IF((9&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(9&gt;=1,9&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(9=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D52" s="17">
+        <f>(B52-$B$5*C52)/((1+$B$6)^9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B53" s="17">
+        <f>(IF(10=1,Calculator!$D$9+Calculator!$D$13*Calculator!$D$14,0))+(IF((10&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(10-1),0))+(IF((10&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0))</f>
+        <v/>
+      </c>
+      <c r="C53" s="17">
+        <f>((IF((10&lt;=Calculator!$B$5),Calculator!$D$10*(1+Calculator!$D$11)^(10-1),0))+(IF((10&lt;=Calculator!$B$5),Calculator!$D$12*Calculator!$B$6,0)))+(IF(AND(10&gt;=1,10&lt;=$B$7),Calculator!$D$9*$B$10/$B$7,0))+(IF(10=1,Calculator!$D$9*(1-$B$10)+Calculator!$D$13*Calculator!$D$14,0))</f>
+        <v/>
+      </c>
+      <c r="D53" s="17">
+        <f>(B53-$B$5*C53)/((1+$B$6)^10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>NPV of after-tax cost</t>
+        </is>
+      </c>
+      <c r="B54" s="17">
+        <f>SUM(B44:B53)</f>
+        <v/>
+      </c>
+      <c r="C54" s="33" t="inlineStr">
+        <is>
+          <t>(nominal cash &lt;-)</t>
+        </is>
+      </c>
+      <c r="D54" s="34">
+        <f>SUM(D44:D53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="n"/>
+      <c r="B57" s="12" t="n"/>
+      <c r="C57" s="12" t="n"/>
+      <c r="D57" s="12" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>Nominal 5-yr cash ($)</t>
+        </is>
+      </c>
+      <c r="B58" s="17">
+        <f>B26</f>
+        <v/>
+      </c>
+      <c r="C58" s="17">
+        <f>B40</f>
+        <v/>
+      </c>
+      <c r="D58" s="17">
+        <f>B54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>After-tax NPV ($)</t>
+        </is>
+      </c>
+      <c r="B59" s="34">
+        <f>D26</f>
+        <v/>
+      </c>
+      <c r="C59" s="34">
+        <f>D40</f>
+        <v/>
+      </c>
+      <c r="D59" s="34">
+        <f>D54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="39" t="inlineStr">
+        <is>
+          <t>Lowest after-tax NPV</t>
+        </is>
+      </c>
+      <c r="B60" s="22">
+        <f>INDEX({"BUILD","BUY","AUTOMATE"},MATCH(MIN(B59:D59),B59:D59,0))</f>
+        <v/>
+      </c>
+      <c r="C60" s="23" t="n"/>
+      <c r="D60" s="24" t="n"/>
+    </row>
+    <row r="62" ht="56" customHeight="1">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>NOT TAX ADVICE. Section 174, bonus depreciation, and capitalization rules change with legislation and vary by jurisdiction and company. Every tax assumption above is an editable blue cell with an illustrative default. Confirm treatment with your finance and tax team. The after-tax NPV, not the nominal cash, is the number most finance teams decide on.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>